<commit_message>
Draft responses for majority of intermediate report deliverable #1
</commit_message>
<xml_diff>
--- a/knowledge/models/capstone_stakeholder_assessment.xlsx
+++ b/knowledge/models/capstone_stakeholder_assessment.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1BAA5E0-5694-46A6-9BBC-76FDDB98A761}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7770" yWindow="0" windowWidth="31080" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="380" yWindow="380" windowWidth="21600" windowHeight="12670" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Stakeholder Assessment" sheetId="1" r:id="rId1"/>
@@ -1105,7 +1105,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -1116,13 +1116,12 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1416,9 +1415,9 @@
     <col min="6" max="6" width="41" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="20.08203125" customWidth="1"/>
     <col min="8" max="8" width="19.4140625" customWidth="1"/>
-    <col min="9" max="9" width="29.1640625" style="6" customWidth="1"/>
+    <col min="9" max="9" width="29.1640625" customWidth="1"/>
     <col min="10" max="10" width="21.58203125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="58.83203125" style="6" customWidth="1"/>
+    <col min="11" max="11" width="58.83203125" customWidth="1"/>
     <col min="12" max="12" width="14.5" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="24.08203125" bestFit="1" customWidth="1"/>
   </cols>
@@ -1448,13 +1447,13 @@
       <c r="H1" s="1" t="s">
         <v>336</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="I1" s="4" t="s">
         <v>6</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="K1" s="4" t="s">
         <v>8</v>
       </c>
       <c r="L1" s="1" t="s">
@@ -1489,13 +1488,13 @@
       <c r="H2" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="I2" s="6" t="s">
+      <c r="I2" t="s">
         <v>18</v>
       </c>
       <c r="J2" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K2" s="6" t="s">
+      <c r="K2" t="s">
         <v>20</v>
       </c>
       <c r="L2" s="2">
@@ -1532,13 +1531,13 @@
       <c r="H3" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="I3" s="6" t="s">
+      <c r="I3" t="s">
         <v>27</v>
       </c>
       <c r="J3" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="K3" s="6" t="s">
+      <c r="K3" t="s">
         <v>29</v>
       </c>
       <c r="L3" s="2">
@@ -1575,13 +1574,13 @@
       <c r="H4" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="I4" s="6" t="s">
+      <c r="I4" t="s">
         <v>35</v>
       </c>
       <c r="J4" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="K4" s="6" t="s">
+      <c r="K4" t="s">
         <v>36</v>
       </c>
       <c r="L4" s="2">
@@ -1593,7 +1592,7 @@
         <v>Boundary input / omit</v>
       </c>
     </row>
-    <row r="5" spans="1:13" hidden="1">
+    <row r="5" spans="1:13" ht="28" hidden="1">
       <c r="A5" s="2" t="s">
         <v>11</v>
       </c>
@@ -1618,13 +1617,13 @@
       <c r="H5" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="I5" s="6" t="s">
+      <c r="I5" t="s">
         <v>41</v>
       </c>
       <c r="J5" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="K5" s="6" t="s">
+      <c r="K5" t="s">
         <v>42</v>
       </c>
       <c r="L5" s="2">
@@ -1636,7 +1635,7 @@
         <v>Boundary input / omit</v>
       </c>
     </row>
-    <row r="6" spans="1:13" ht="28">
+    <row r="6" spans="1:13">
       <c r="A6" s="2" t="s">
         <v>11</v>
       </c>
@@ -1661,13 +1660,13 @@
       <c r="H6" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="I6" s="6" t="s">
+      <c r="I6" t="s">
         <v>48</v>
       </c>
       <c r="J6" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="K6" s="6" t="s">
+      <c r="K6" t="s">
         <v>50</v>
       </c>
       <c r="L6" s="2">
@@ -1704,13 +1703,13 @@
       <c r="H7" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="I7" s="6" t="s">
+      <c r="I7" t="s">
         <v>55</v>
       </c>
       <c r="J7" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="K7" s="6" t="s">
+      <c r="K7" t="s">
         <v>56</v>
       </c>
       <c r="L7" s="2">
@@ -1747,13 +1746,13 @@
       <c r="H8" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="I8" s="6" t="s">
+      <c r="I8" t="s">
         <v>61</v>
       </c>
       <c r="J8" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="K8" s="6" t="s">
+      <c r="K8" t="s">
         <v>62</v>
       </c>
       <c r="L8" s="2">
@@ -1790,13 +1789,13 @@
       <c r="H9" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="I9" s="6" t="s">
+      <c r="I9" t="s">
         <v>67</v>
       </c>
       <c r="J9" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K9" s="6" t="s">
+      <c r="K9" t="s">
         <v>68</v>
       </c>
       <c r="L9" s="2">
@@ -1833,13 +1832,13 @@
       <c r="H10" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I10" s="6" t="s">
+      <c r="I10" t="s">
         <v>75</v>
       </c>
       <c r="J10" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K10" s="6" t="s">
+      <c r="K10" t="s">
         <v>76</v>
       </c>
       <c r="L10" s="2">
@@ -1876,13 +1875,13 @@
       <c r="H11" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I11" s="6" t="s">
+      <c r="I11" t="s">
         <v>81</v>
       </c>
       <c r="J11" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K11" s="6" t="s">
+      <c r="K11" t="s">
         <v>82</v>
       </c>
       <c r="L11" s="2">
@@ -1919,13 +1918,13 @@
       <c r="H12" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I12" s="6" t="s">
+      <c r="I12" t="s">
         <v>86</v>
       </c>
       <c r="J12" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K12" s="6" t="s">
+      <c r="K12" t="s">
         <v>87</v>
       </c>
       <c r="L12" s="2">
@@ -1962,13 +1961,13 @@
       <c r="H13" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="I13" s="6" t="s">
+      <c r="I13" t="s">
         <v>92</v>
       </c>
       <c r="J13" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="K13" s="6" t="s">
+      <c r="K13" t="s">
         <v>93</v>
       </c>
       <c r="L13" s="2">
@@ -2005,13 +2004,13 @@
       <c r="H14" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="I14" s="6" t="s">
+      <c r="I14" t="s">
         <v>99</v>
       </c>
       <c r="J14" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K14" s="6" t="s">
+      <c r="K14" t="s">
         <v>100</v>
       </c>
       <c r="L14" s="2">
@@ -2048,13 +2047,13 @@
       <c r="H15" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I15" s="6" t="s">
+      <c r="I15" t="s">
         <v>105</v>
       </c>
       <c r="J15" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K15" s="6" t="s">
+      <c r="K15" t="s">
         <v>106</v>
       </c>
       <c r="L15" s="2">
@@ -2091,13 +2090,13 @@
       <c r="H16" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="I16" s="6" t="s">
+      <c r="I16" t="s">
         <v>111</v>
       </c>
       <c r="J16" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="K16" s="6" t="s">
+      <c r="K16" t="s">
         <v>112</v>
       </c>
       <c r="L16" s="2">
@@ -2134,13 +2133,13 @@
       <c r="H17" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="I17" s="6" t="s">
+      <c r="I17" t="s">
         <v>118</v>
       </c>
       <c r="J17" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="K17" s="6" t="s">
+      <c r="K17" t="s">
         <v>119</v>
       </c>
       <c r="L17" s="2">
@@ -2177,13 +2176,13 @@
       <c r="H18" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="I18" s="6" t="s">
+      <c r="I18" t="s">
         <v>125</v>
       </c>
       <c r="J18" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="K18" s="6" t="s">
+      <c r="K18" t="s">
         <v>126</v>
       </c>
       <c r="L18" s="2">
@@ -2220,13 +2219,13 @@
       <c r="H19" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="I19" s="6" t="s">
+      <c r="I19" t="s">
         <v>131</v>
       </c>
       <c r="J19" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="K19" s="6" t="s">
+      <c r="K19" t="s">
         <v>132</v>
       </c>
       <c r="L19" s="2">
@@ -2263,13 +2262,13 @@
       <c r="H20" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I20" s="6" t="s">
+      <c r="I20" t="s">
         <v>137</v>
       </c>
       <c r="J20" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="K20" s="6" t="s">
+      <c r="K20" t="s">
         <v>138</v>
       </c>
       <c r="L20" s="2">
@@ -2306,13 +2305,13 @@
       <c r="H21" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I21" s="6" t="s">
+      <c r="I21" t="s">
         <v>143</v>
       </c>
       <c r="J21" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K21" s="6" t="s">
+      <c r="K21" t="s">
         <v>144</v>
       </c>
       <c r="L21" s="2">
@@ -2349,13 +2348,13 @@
       <c r="H22" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I22" s="6" t="s">
+      <c r="I22" t="s">
         <v>149</v>
       </c>
       <c r="J22" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="K22" s="6" t="s">
+      <c r="K22" t="s">
         <v>150</v>
       </c>
       <c r="L22" s="2">
@@ -2392,13 +2391,13 @@
       <c r="H23" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I23" s="6" t="s">
+      <c r="I23" t="s">
         <v>156</v>
       </c>
       <c r="J23" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K23" s="6" t="s">
+      <c r="K23" t="s">
         <v>157</v>
       </c>
       <c r="L23" s="2">
@@ -2435,13 +2434,13 @@
       <c r="H24" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I24" s="6" t="s">
+      <c r="I24" t="s">
         <v>163</v>
       </c>
       <c r="J24" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="K24" s="6" t="s">
+      <c r="K24" t="s">
         <v>164</v>
       </c>
       <c r="L24" s="2">
@@ -2478,13 +2477,13 @@
       <c r="H25" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I25" s="6" t="s">
+      <c r="I25" t="s">
         <v>169</v>
       </c>
       <c r="J25" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K25" s="6" t="s">
+      <c r="K25" t="s">
         <v>170</v>
       </c>
       <c r="L25" s="2">
@@ -2521,13 +2520,13 @@
       <c r="H26" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="I26" s="6" t="s">
+      <c r="I26" t="s">
         <v>175</v>
       </c>
       <c r="J26" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="K26" s="6" t="s">
+      <c r="K26" t="s">
         <v>176</v>
       </c>
       <c r="L26" s="2">
@@ -2564,13 +2563,13 @@
       <c r="H27" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="I27" s="6" t="s">
+      <c r="I27" t="s">
         <v>182</v>
       </c>
       <c r="J27" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="K27" s="6" t="s">
+      <c r="K27" t="s">
         <v>183</v>
       </c>
       <c r="L27" s="2">
@@ -2607,13 +2606,13 @@
       <c r="H28" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I28" s="6" t="s">
+      <c r="I28" t="s">
         <v>188</v>
       </c>
       <c r="J28" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="K28" s="6" t="s">
+      <c r="K28" t="s">
         <v>189</v>
       </c>
       <c r="L28" s="2">
@@ -2650,13 +2649,13 @@
       <c r="H29" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="I29" s="6" t="s">
+      <c r="I29" t="s">
         <v>194</v>
       </c>
       <c r="J29" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="K29" s="6" t="s">
+      <c r="K29" t="s">
         <v>195</v>
       </c>
       <c r="L29" s="2">
@@ -2668,7 +2667,7 @@
         <v>Boundary input / omit</v>
       </c>
     </row>
-    <row r="30" spans="1:13" hidden="1">
+    <row r="30" spans="1:13" ht="28" hidden="1">
       <c r="A30" s="2" t="s">
         <v>196</v>
       </c>
@@ -2693,13 +2692,13 @@
       <c r="H30" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="I30" s="6" t="s">
+      <c r="I30" t="s">
         <v>202</v>
       </c>
       <c r="J30" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="K30" s="6" t="s">
+      <c r="K30" t="s">
         <v>203</v>
       </c>
       <c r="L30" s="2">
@@ -2736,13 +2735,13 @@
       <c r="H31" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="I31" s="6" t="s">
+      <c r="I31" t="s">
         <v>209</v>
       </c>
       <c r="J31" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="K31" s="6" t="s">
+      <c r="K31" t="s">
         <v>210</v>
       </c>
       <c r="L31" s="2">
@@ -2779,13 +2778,13 @@
       <c r="H32" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="I32" s="6" t="s">
+      <c r="I32" t="s">
         <v>216</v>
       </c>
       <c r="J32" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="K32" s="6" t="s">
+      <c r="K32" t="s">
         <v>217</v>
       </c>
       <c r="L32" s="2">
@@ -2822,13 +2821,13 @@
       <c r="H33" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I33" s="6" t="s">
+      <c r="I33" t="s">
         <v>221</v>
       </c>
       <c r="J33" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K33" s="6" t="s">
+      <c r="K33" t="s">
         <v>222</v>
       </c>
       <c r="L33" s="2">
@@ -2836,7 +2835,7 @@
         <v>5</v>
       </c>
       <c r="M33" s="2" t="str">
-        <f t="shared" ref="M33:M64" si="3">IF(L33&gt;=5,"Standalone",IF(L33&gt;=3,"Consider / Consolidate","Boundary input / omit"))</f>
+        <f t="shared" ref="M33:M49" si="3">IF(L33&gt;=5,"Standalone",IF(L33&gt;=3,"Consider / Consolidate","Boundary input / omit"))</f>
         <v>Standalone</v>
       </c>
     </row>
@@ -2865,13 +2864,13 @@
       <c r="H34" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I34" s="6" t="s">
+      <c r="I34" t="s">
         <v>228</v>
       </c>
       <c r="J34" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K34" s="6" t="s">
+      <c r="K34" t="s">
         <v>229</v>
       </c>
       <c r="L34" s="2">
@@ -2908,13 +2907,13 @@
       <c r="H35" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="I35" s="6" t="s">
+      <c r="I35" t="s">
         <v>234</v>
       </c>
       <c r="J35" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="K35" s="6" t="s">
+      <c r="K35" t="s">
         <v>235</v>
       </c>
       <c r="L35" s="2">
@@ -2951,13 +2950,13 @@
       <c r="H36" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="I36" s="6" t="s">
+      <c r="I36" t="s">
         <v>240</v>
       </c>
       <c r="J36" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="K36" s="6" t="s">
+      <c r="K36" t="s">
         <v>241</v>
       </c>
       <c r="L36" s="2">
@@ -2969,7 +2968,7 @@
         <v>Boundary input / omit</v>
       </c>
     </row>
-    <row r="37" spans="1:13" hidden="1">
+    <row r="37" spans="1:13" ht="28" hidden="1">
       <c r="A37" s="2" t="s">
         <v>196</v>
       </c>
@@ -2994,13 +2993,13 @@
       <c r="H37" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="I37" s="6" t="s">
+      <c r="I37" t="s">
         <v>246</v>
       </c>
       <c r="J37" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="K37" s="6" t="s">
+      <c r="K37" t="s">
         <v>247</v>
       </c>
       <c r="L37" s="2">
@@ -3037,13 +3036,13 @@
       <c r="H38" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="I38" s="6" t="s">
+      <c r="I38" t="s">
         <v>253</v>
       </c>
       <c r="J38" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="K38" s="6" t="s">
+      <c r="K38" t="s">
         <v>254</v>
       </c>
       <c r="L38" s="2">
@@ -3080,13 +3079,13 @@
       <c r="H39" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="I39" s="6" t="s">
+      <c r="I39" t="s">
         <v>259</v>
       </c>
       <c r="J39" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="K39" s="6" t="s">
+      <c r="K39" t="s">
         <v>260</v>
       </c>
       <c r="L39" s="2">
@@ -3123,13 +3122,13 @@
       <c r="H40" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="I40" s="6" t="s">
+      <c r="I40" t="s">
         <v>265</v>
       </c>
       <c r="J40" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="K40" s="6" t="s">
+      <c r="K40" t="s">
         <v>266</v>
       </c>
       <c r="L40" s="2">
@@ -3166,13 +3165,13 @@
       <c r="H41" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="I41" s="6" t="s">
+      <c r="I41" t="s">
         <v>271</v>
       </c>
       <c r="J41" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="K41" s="6" t="s">
+      <c r="K41" t="s">
         <v>272</v>
       </c>
       <c r="L41" s="2">
@@ -3209,13 +3208,13 @@
       <c r="H42" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="I42" s="6" t="s">
+      <c r="I42" t="s">
         <v>277</v>
       </c>
       <c r="J42" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="K42" s="6" t="s">
+      <c r="K42" t="s">
         <v>278</v>
       </c>
       <c r="L42" s="2">
@@ -3252,13 +3251,13 @@
       <c r="H43" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="I43" s="6" t="s">
+      <c r="I43" t="s">
         <v>283</v>
       </c>
       <c r="J43" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="K43" s="6" t="s">
+      <c r="K43" t="s">
         <v>284</v>
       </c>
       <c r="L43" s="2">
@@ -3295,13 +3294,13 @@
       <c r="H44" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I44" s="6" t="s">
+      <c r="I44" t="s">
         <v>290</v>
       </c>
       <c r="J44" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="K44" s="6" t="s">
+      <c r="K44" t="s">
         <v>291</v>
       </c>
       <c r="L44" s="2">
@@ -3338,13 +3337,13 @@
       <c r="H45" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I45" s="6" t="s">
+      <c r="I45" t="s">
         <v>295</v>
       </c>
       <c r="J45" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K45" s="6" t="s">
+      <c r="K45" t="s">
         <v>296</v>
       </c>
       <c r="L45" s="2">
@@ -3381,13 +3380,13 @@
       <c r="H46" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="I46" s="6" t="s">
+      <c r="I46" t="s">
         <v>301</v>
       </c>
       <c r="J46" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="K46" s="6" t="s">
+      <c r="K46" t="s">
         <v>302</v>
       </c>
       <c r="L46" s="2">
@@ -3424,13 +3423,13 @@
       <c r="H47" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I47" s="6" t="s">
+      <c r="I47" t="s">
         <v>308</v>
       </c>
       <c r="J47" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="K47" s="6" t="s">
+      <c r="K47" t="s">
         <v>337</v>
       </c>
       <c r="L47" s="2">
@@ -3467,13 +3466,13 @@
       <c r="H48" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="I48" s="6" t="s">
+      <c r="I48" t="s">
         <v>313</v>
       </c>
       <c r="J48" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="K48" s="6" t="s">
+      <c r="K48" t="s">
         <v>314</v>
       </c>
       <c r="L48" s="2">
@@ -3510,13 +3509,13 @@
       <c r="H49" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="I49" s="6" t="s">
+      <c r="I49" t="s">
         <v>319</v>
       </c>
       <c r="J49" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="K49" s="6" t="s">
+      <c r="K49" t="s">
         <v>320</v>
       </c>
       <c r="L49" s="2">
@@ -3565,10 +3564,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="20">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="5" t="s">
         <v>321</v>
       </c>
-      <c r="B1" s="4"/>
+      <c r="B1" s="5"/>
     </row>
     <row r="2" spans="1:2" ht="28">
       <c r="A2" s="2" t="s">

</xml_diff>

<commit_message>
Update NAS project scope, evidence, and planning records
</commit_message>
<xml_diff>
--- a/knowledge/models/capstone_stakeholder_assessment.xlsx
+++ b/knowledge/models/capstone_stakeholder_assessment.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\repos\capstone_isd\knowledge\models\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1BAA5E0-5694-46A6-9BBC-76FDDB98A761}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDDBC960-B364-4070-A69B-909268084EE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="380" yWindow="380" windowWidth="21600" windowHeight="12670" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="840" yWindow="0" windowWidth="29655" windowHeight="20985" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Stakeholder Assessment" sheetId="1" r:id="rId1"/>
     <sheet name="Decision Guide" sheetId="2" r:id="rId2"/>
+    <sheet name="system definition decisions" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -32,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="558" uniqueCount="338">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="665" uniqueCount="399">
   <si>
     <t>PESTLE Domain</t>
   </si>
@@ -1046,16 +1047,220 @@
   </si>
   <si>
     <t>Consolidate with Airports.</t>
+  </si>
+  <si>
+    <t>capability allocated to operators/ATM</t>
+  </si>
+  <si>
+    <t>absorb/abstract</t>
+  </si>
+  <si>
+    <t>Decision Support</t>
+  </si>
+  <si>
+    <t>context constraint</t>
+  </si>
+  <si>
+    <t>Maintenance Suppliers</t>
+  </si>
+  <si>
+    <t>Decide behavior of aircraft and transport information from plan to enaction.</t>
+  </si>
+  <si>
+    <t>Crew</t>
+  </si>
+  <si>
+    <t>Military</t>
+  </si>
+  <si>
+    <t>Modelling may influence KPIs sufficient to change decisions and can't be absorbed into another in a consistent way (regulatory/legal, or otherwise)</t>
+  </si>
+  <si>
+    <t>decided either externally, so they're a constraint, or is sufficiently outside the scope of the project (e.g. airspace region definitions and how allocation determines congestion &amp; workload).</t>
+  </si>
+  <si>
+    <t>Infra / Airspace Resources</t>
+  </si>
+  <si>
+    <t>Info Systems</t>
+  </si>
+  <si>
+    <t>Encompasses all sub-systems and is the 'final entity' whose behavior determines KPIs</t>
+  </si>
+  <si>
+    <t>Aircraft</t>
+  </si>
+  <si>
+    <t>A/C Systems</t>
+  </si>
+  <si>
+    <t>Operators decide operations and encompass Airlines and other actors, though not all have the same internal composition</t>
+  </si>
+  <si>
+    <t>Operators</t>
+  </si>
+  <si>
+    <t>Airline</t>
+  </si>
+  <si>
+    <t>Flight Ops</t>
+  </si>
+  <si>
+    <t>Airports represent their own pseudo-ecosystem, which operates largely independently, but which has a great effect on KPIs</t>
+  </si>
+  <si>
+    <t>Airport(s)</t>
+  </si>
+  <si>
+    <t>Airport</t>
+  </si>
+  <si>
+    <t>Airport Ops</t>
+  </si>
+  <si>
+    <t>A generic term applied to all organizations and divisions responsible for actively directing traffic.</t>
+  </si>
+  <si>
+    <t>ATC/ANSP</t>
+  </si>
+  <si>
+    <t>ATC</t>
+  </si>
+  <si>
+    <t>Airspace Management</t>
+  </si>
+  <si>
+    <t>Regulatory / Legal</t>
+  </si>
+  <si>
+    <t>Envinronmental/Societal</t>
+  </si>
+  <si>
+    <t>Governance</t>
+  </si>
+  <si>
+    <t>Rationale</t>
+  </si>
+  <si>
+    <t>Decision</t>
+  </si>
+  <si>
+    <t>Stakeholder Ontology</t>
+  </si>
+  <si>
+    <t>SOI</t>
+  </si>
+  <si>
+    <t>Candidate Systems</t>
+  </si>
+  <si>
+    <t>could be incoporated in operators, but I will keep that Part 121 scheduled passenger airlines due to the complexity of their operations and that they represent the vast majority of air traffic.</t>
+  </si>
+  <si>
+    <t>Project Action</t>
+  </si>
+  <si>
+    <t>Boundary Actor</t>
+  </si>
+  <si>
+    <t>Modelled System</t>
+  </si>
+  <si>
+    <t>Absorbed</t>
+  </si>
+  <si>
+    <t>boundary actor</t>
+  </si>
+  <si>
+    <t>Impact can be modelled as part of airline operations; Likely limited to cost parameter and not influencing KPIs dynamically.</t>
+  </si>
+  <si>
+    <t>ATC / ANSP</t>
+  </si>
+  <si>
+    <t>info exchange will be an abstraction/background-level info. "data"/"info" will be exchanged between systems and where channels/mechanisms are important/relevant, I will add a decision activity to specify through which channel.</t>
+  </si>
+  <si>
+    <t>Flight Crew</t>
+  </si>
+  <si>
+    <t>it encompasses the other two and is the channel(s) through which all social organizations will influence KPIs, but they aren't modified by the decisions I believe I'll be exploring.  regulation is held fixed in the baseline, with sensitivity sweeps as an optional extension.</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>Refined:</t>
+  </si>
+  <si>
+    <t>Candidate</t>
+  </si>
+  <si>
+    <t>Revised rationale</t>
+  </si>
+  <si>
+    <t>Sets the legal, regulatory, and policy context through which societal and environmental objectives influence the modeled systems. Governance is held fixed in the baseline because the decisions under study do not modify it; regulatory sensitivity sweeps are an optional extension.</t>
+  </si>
+  <si>
+    <t>Part 121 scheduled passenger operators are modeled because their dispatch, scheduling, routing, and recovery decisions are dynamically coupled to RPM, cost, safety, workload, and schedule-performance measures. Other operators are represented only as background traffic where their presence materially affects a selected KPI.</t>
+  </si>
+  <si>
+    <t>Use the passenger rationale above.</t>
+  </si>
+  <si>
+    <t>Military operations are outside the modeled operator population. Where military traffic or special-use airspace materially affects civil safety, capacity, or workload, it is represented as an external constraint or background scenario input rather than decomposed as an operator system.</t>
+  </si>
+  <si>
+    <t>Context Constraint</t>
+  </si>
+  <si>
+    <t>Supplier-side maintenance cost, availability, and turnaround effects are represented as exogenous parameters. Airline maintenance planning, deferral, and release decisions remain part of Flight Operations.</t>
+  </si>
+  <si>
+    <t>Airspace structure, navigation infrastructure, and shared resources are externally determined constraints in the baseline. Their effects may be varied parametrically when testing congestion, workload, safety, or capacity sensitivity.</t>
+  </si>
+  <si>
+    <t>Absorbed / Abstracted</t>
+  </si>
+  <si>
+    <t>Information is modeled as exchanges between systems. The specific channel is represented only when channel reliability, latency, or capability changes the decision or KPI.</t>
+  </si>
+  <si>
+    <t>Decision-support capability is allocated to the operator or ATM context rather than treated as an independent stakeholder system; its recommendations and information dependencies remain modelable.</t>
+  </si>
+  <si>
+    <t>Include an entity as a modeled system when it has distinct decision authority or execution behavior that is dynamically coupled to in-scope decisions and materially affects selected KPIs. Represent an entity as a boundary actor when it supplies objectives, demand, feedback, or constraints without being decomposed as a decision mechanism. Represent exogenous influences as parameters or scenario inputs.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <b/>
@@ -1074,8 +1279,16 @@
       <sz val="11"/>
       <name val="Carlito"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1092,8 +1305,26 @@
         <fgColor rgb="FFD9EAF7"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1101,30 +1332,77 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 2" xfId="1" xr:uid="{3EB05A31-C3B2-4E4E-8A77-433CC7A006A5}"/>
   </cellStyles>
   <dxfs count="6">
     <dxf>
@@ -1181,15 +1459,7 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="StakeholderAssessment" displayName="StakeholderAssessment" ref="A1:M49" totalsRowShown="0">
-  <autoFilter ref="A1:M49" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}">
-    <filterColumn colId="11">
-      <filters>
-        <filter val="3"/>
-        <filter val="4"/>
-        <filter val="5"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:M49" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}"/>
   <tableColumns count="13">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="PESTLE Domain"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Stakeholder"/>
@@ -1506,7 +1776,7 @@
         <v>Consider / Consolidate</v>
       </c>
     </row>
-    <row r="3" spans="1:13" ht="14" hidden="1" customHeight="1">
+    <row r="3" spans="1:13" ht="14" customHeight="1">
       <c r="A3" s="2" t="s">
         <v>11</v>
       </c>
@@ -1549,7 +1819,7 @@
         <v>Boundary input / omit</v>
       </c>
     </row>
-    <row r="4" spans="1:13" hidden="1">
+    <row r="4" spans="1:13">
       <c r="A4" s="2" t="s">
         <v>11</v>
       </c>
@@ -1592,7 +1862,7 @@
         <v>Boundary input / omit</v>
       </c>
     </row>
-    <row r="5" spans="1:13" ht="28" hidden="1">
+    <row r="5" spans="1:13" ht="28">
       <c r="A5" s="2" t="s">
         <v>11</v>
       </c>
@@ -1678,7 +1948,7 @@
         <v>Consider / Consolidate</v>
       </c>
     </row>
-    <row r="7" spans="1:13" hidden="1">
+    <row r="7" spans="1:13">
       <c r="A7" s="2" t="s">
         <v>11</v>
       </c>
@@ -1721,7 +1991,7 @@
         <v>Boundary input / omit</v>
       </c>
     </row>
-    <row r="8" spans="1:13" hidden="1">
+    <row r="8" spans="1:13">
       <c r="A8" s="2" t="s">
         <v>11</v>
       </c>
@@ -1936,7 +2206,7 @@
         <v>Standalone</v>
       </c>
     </row>
-    <row r="13" spans="1:13" ht="28" hidden="1">
+    <row r="13" spans="1:13" ht="28">
       <c r="A13" s="2" t="s">
         <v>69</v>
       </c>
@@ -2065,7 +2335,7 @@
         <v>Standalone</v>
       </c>
     </row>
-    <row r="16" spans="1:13" hidden="1">
+    <row r="16" spans="1:13">
       <c r="A16" s="2" t="s">
         <v>69</v>
       </c>
@@ -2108,7 +2378,7 @@
         <v>Boundary input / omit</v>
       </c>
     </row>
-    <row r="17" spans="1:13" hidden="1">
+    <row r="17" spans="1:13">
       <c r="A17" s="2" t="s">
         <v>69</v>
       </c>
@@ -2151,7 +2421,7 @@
         <v>Boundary input / omit</v>
       </c>
     </row>
-    <row r="18" spans="1:13" hidden="1">
+    <row r="18" spans="1:13">
       <c r="A18" s="2" t="s">
         <v>69</v>
       </c>
@@ -2237,7 +2507,7 @@
         <v>Consider / Consolidate</v>
       </c>
     </row>
-    <row r="20" spans="1:13" hidden="1">
+    <row r="20" spans="1:13">
       <c r="A20" s="2" t="s">
         <v>69</v>
       </c>
@@ -2323,7 +2593,7 @@
         <v>Consider / Consolidate</v>
       </c>
     </row>
-    <row r="22" spans="1:13" hidden="1">
+    <row r="22" spans="1:13">
       <c r="A22" s="2" t="s">
         <v>145</v>
       </c>
@@ -2409,7 +2679,7 @@
         <v>Consider / Consolidate</v>
       </c>
     </row>
-    <row r="24" spans="1:13" hidden="1">
+    <row r="24" spans="1:13">
       <c r="A24" s="2" t="s">
         <v>145</v>
       </c>
@@ -2495,7 +2765,7 @@
         <v>Consider / Consolidate</v>
       </c>
     </row>
-    <row r="26" spans="1:13" hidden="1">
+    <row r="26" spans="1:13">
       <c r="A26" s="2" t="s">
         <v>145</v>
       </c>
@@ -2538,7 +2808,7 @@
         <v>Boundary input / omit</v>
       </c>
     </row>
-    <row r="27" spans="1:13" hidden="1">
+    <row r="27" spans="1:13">
       <c r="A27" s="2" t="s">
         <v>145</v>
       </c>
@@ -2624,7 +2894,7 @@
         <v>Consider / Consolidate</v>
       </c>
     </row>
-    <row r="29" spans="1:13" hidden="1">
+    <row r="29" spans="1:13">
       <c r="A29" s="2" t="s">
         <v>145</v>
       </c>
@@ -2667,7 +2937,7 @@
         <v>Boundary input / omit</v>
       </c>
     </row>
-    <row r="30" spans="1:13" ht="28" hidden="1">
+    <row r="30" spans="1:13" ht="28">
       <c r="A30" s="2" t="s">
         <v>196</v>
       </c>
@@ -2710,7 +2980,7 @@
         <v>Boundary input / omit</v>
       </c>
     </row>
-    <row r="31" spans="1:13" hidden="1">
+    <row r="31" spans="1:13">
       <c r="A31" s="2" t="s">
         <v>196</v>
       </c>
@@ -2882,7 +3152,7 @@
         <v>Standalone</v>
       </c>
     </row>
-    <row r="35" spans="1:13" ht="28" hidden="1">
+    <row r="35" spans="1:13" ht="28">
       <c r="A35" s="2" t="s">
         <v>196</v>
       </c>
@@ -2925,7 +3195,7 @@
         <v>Boundary input / omit</v>
       </c>
     </row>
-    <row r="36" spans="1:13" hidden="1">
+    <row r="36" spans="1:13">
       <c r="A36" s="2" t="s">
         <v>196</v>
       </c>
@@ -2968,7 +3238,7 @@
         <v>Boundary input / omit</v>
       </c>
     </row>
-    <row r="37" spans="1:13" ht="28" hidden="1">
+    <row r="37" spans="1:13" ht="28">
       <c r="A37" s="2" t="s">
         <v>196</v>
       </c>
@@ -3011,7 +3281,7 @@
         <v>Boundary input / omit</v>
       </c>
     </row>
-    <row r="38" spans="1:13" hidden="1">
+    <row r="38" spans="1:13">
       <c r="A38" s="2" t="s">
         <v>248</v>
       </c>
@@ -3054,7 +3324,7 @@
         <v>Boundary input / omit</v>
       </c>
     </row>
-    <row r="39" spans="1:13" hidden="1">
+    <row r="39" spans="1:13">
       <c r="A39" s="2" t="s">
         <v>248</v>
       </c>
@@ -3097,7 +3367,7 @@
         <v>Boundary input / omit</v>
       </c>
     </row>
-    <row r="40" spans="1:13" hidden="1">
+    <row r="40" spans="1:13">
       <c r="A40" s="2" t="s">
         <v>248</v>
       </c>
@@ -3140,7 +3410,7 @@
         <v>Boundary input / omit</v>
       </c>
     </row>
-    <row r="41" spans="1:13" hidden="1">
+    <row r="41" spans="1:13">
       <c r="A41" s="2" t="s">
         <v>248</v>
       </c>
@@ -3183,7 +3453,7 @@
         <v>Boundary input / omit</v>
       </c>
     </row>
-    <row r="42" spans="1:13" hidden="1">
+    <row r="42" spans="1:13">
       <c r="A42" s="2" t="s">
         <v>248</v>
       </c>
@@ -3226,7 +3496,7 @@
         <v>Boundary input / omit</v>
       </c>
     </row>
-    <row r="43" spans="1:13" hidden="1">
+    <row r="43" spans="1:13">
       <c r="A43" s="2" t="s">
         <v>248</v>
       </c>
@@ -3355,7 +3625,7 @@
         <v>Consider / Consolidate</v>
       </c>
     </row>
-    <row r="46" spans="1:13" hidden="1">
+    <row r="46" spans="1:13">
       <c r="A46" s="2" t="s">
         <v>285</v>
       </c>
@@ -3398,7 +3668,7 @@
         <v>Boundary input / omit</v>
       </c>
     </row>
-    <row r="47" spans="1:13" hidden="1">
+    <row r="47" spans="1:13">
       <c r="A47" s="2" t="s">
         <v>285</v>
       </c>
@@ -3441,7 +3711,7 @@
         <v>Boundary input / omit</v>
       </c>
     </row>
-    <row r="48" spans="1:13" hidden="1">
+    <row r="48" spans="1:13">
       <c r="A48" s="2" t="s">
         <v>285</v>
       </c>
@@ -3484,7 +3754,7 @@
         <v>Boundary input / omit</v>
       </c>
     </row>
-    <row r="49" spans="1:13" hidden="1">
+    <row r="49" spans="1:13">
       <c r="A49" s="2" t="s">
         <v>285</v>
       </c>
@@ -3564,10 +3834,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="20">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="13" t="s">
         <v>321</v>
       </c>
-      <c r="B1" s="5"/>
+      <c r="B1" s="13"/>
     </row>
     <row r="2" spans="1:2" ht="28">
       <c r="A2" s="2" t="s">
@@ -3639,4 +3909,391 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1CD39BF1-CAA2-4876-A3AC-3E5F1F00D9DB}">
+  <dimension ref="A1:F31"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
+  <cols>
+    <col min="1" max="3" width="21.6640625" style="5" customWidth="1"/>
+    <col min="4" max="4" width="16.75" style="5" customWidth="1"/>
+    <col min="5" max="5" width="36.75" style="5" customWidth="1"/>
+    <col min="6" max="6" width="87.75" style="5" customWidth="1"/>
+    <col min="7" max="16384" width="8.6640625" style="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6">
+      <c r="A1" s="9" t="s">
+        <v>372</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>371</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>370</v>
+      </c>
+      <c r="D1" s="9" t="s">
+        <v>369</v>
+      </c>
+      <c r="E1" s="9" t="s">
+        <v>374</v>
+      </c>
+      <c r="F1" s="9" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="43.5">
+      <c r="A2" s="6" t="s">
+        <v>367</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>365</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>366</v>
+      </c>
+      <c r="D2" s="10" t="s">
+        <v>378</v>
+      </c>
+      <c r="E2" s="10" t="s">
+        <v>375</v>
+      </c>
+      <c r="F2" s="14" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3" s="6" t="s">
+        <v>364</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>363</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>362</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>380</v>
+      </c>
+      <c r="E3" s="10" t="s">
+        <v>376</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="29">
+      <c r="A4" s="6" t="s">
+        <v>360</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>359</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>358</v>
+      </c>
+      <c r="E4" s="10" t="s">
+        <v>376</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="29">
+      <c r="A5" s="6" t="s">
+        <v>356</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>354</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>355</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>354</v>
+      </c>
+      <c r="E5" s="10" t="s">
+        <v>376</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
+      <c r="A6" s="6" t="s">
+        <v>352</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>351</v>
+      </c>
+      <c r="C6" s="15" t="s">
+        <v>384</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>351</v>
+      </c>
+      <c r="E6" s="10" t="s">
+        <v>376</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="43.5">
+      <c r="A7" s="6" t="s">
+        <v>349</v>
+      </c>
+      <c r="B7" s="15" t="s">
+        <v>384</v>
+      </c>
+      <c r="C7" s="15" t="s">
+        <v>384</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>339</v>
+      </c>
+      <c r="E7" s="11" t="s">
+        <v>377</v>
+      </c>
+      <c r="F7" s="11" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="29">
+      <c r="A8" s="6" t="s">
+        <v>348</v>
+      </c>
+      <c r="B8" s="15" t="s">
+        <v>384</v>
+      </c>
+      <c r="C8" s="15" t="s">
+        <v>384</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>341</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>341</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="29">
+      <c r="A9" s="15" t="s">
+        <v>384</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>139</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>139</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>139</v>
+      </c>
+      <c r="E9" s="10" t="s">
+        <v>376</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="29">
+      <c r="A10" s="15" t="s">
+        <v>384</v>
+      </c>
+      <c r="B10" s="15" t="s">
+        <v>384</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>345</v>
+      </c>
+      <c r="D10" s="14" t="s">
+        <v>378</v>
+      </c>
+      <c r="E10" s="14" t="s">
+        <v>378</v>
+      </c>
+      <c r="F10" s="11" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
+      <c r="A11" s="15" t="s">
+        <v>384</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>344</v>
+      </c>
+      <c r="C11" s="12" t="s">
+        <v>382</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>344</v>
+      </c>
+      <c r="E11" s="10" t="s">
+        <v>376</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="29">
+      <c r="A12" s="15" t="s">
+        <v>384</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>342</v>
+      </c>
+      <c r="C12" s="15" t="s">
+        <v>384</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>341</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>341</v>
+      </c>
+      <c r="F12" s="11" t="s">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6">
+      <c r="A13" s="15" t="s">
+        <v>384</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>340</v>
+      </c>
+      <c r="C13" s="15" t="s">
+        <v>384</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>339</v>
+      </c>
+      <c r="E13" s="11" t="s">
+        <v>377</v>
+      </c>
+      <c r="F13" s="5" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="19" spans="4:6">
+      <c r="D19" s="14" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="20" spans="4:6">
+      <c r="D20" s="6" t="s">
+        <v>386</v>
+      </c>
+      <c r="E20" s="6" t="s">
+        <v>374</v>
+      </c>
+      <c r="F20" s="6" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="21" spans="4:6" ht="43.5">
+      <c r="D21" s="6" t="s">
+        <v>367</v>
+      </c>
+      <c r="E21" s="6" t="s">
+        <v>375</v>
+      </c>
+      <c r="F21" s="6" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="22" spans="4:6" ht="43.5">
+      <c r="D22" s="6" t="s">
+        <v>356</v>
+      </c>
+      <c r="E22" s="6" t="s">
+        <v>376</v>
+      </c>
+      <c r="F22" s="6" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="23" spans="4:6">
+      <c r="D23" s="6" t="s">
+        <v>139</v>
+      </c>
+      <c r="E23" s="6" t="s">
+        <v>375</v>
+      </c>
+      <c r="F23" s="6" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="24" spans="4:6" ht="43.5">
+      <c r="D24" s="6" t="s">
+        <v>345</v>
+      </c>
+      <c r="E24" s="6" t="s">
+        <v>375</v>
+      </c>
+      <c r="F24" s="6" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="25" spans="4:6" ht="29">
+      <c r="D25" s="6" t="s">
+        <v>342</v>
+      </c>
+      <c r="E25" s="6" t="s">
+        <v>392</v>
+      </c>
+      <c r="F25" s="6" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="26" spans="4:6" ht="43.5">
+      <c r="D26" s="6" t="s">
+        <v>348</v>
+      </c>
+      <c r="E26" s="6" t="s">
+        <v>392</v>
+      </c>
+      <c r="F26" s="6" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="27" spans="4:6" ht="29">
+      <c r="D27" s="6" t="s">
+        <v>349</v>
+      </c>
+      <c r="E27" s="6" t="s">
+        <v>395</v>
+      </c>
+      <c r="F27" s="6" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="28" spans="4:6" ht="29">
+      <c r="D28" s="6" t="s">
+        <v>340</v>
+      </c>
+      <c r="E28" s="6" t="s">
+        <v>395</v>
+      </c>
+      <c r="F28" s="6" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="31" spans="4:6" ht="58">
+      <c r="E31" s="14"/>
+      <c r="F31" s="14" t="s">
+        <v>398</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>